<commit_message>
Update repo dependency to the latest version of dqLib
</commit_message>
<xml_diff>
--- a/data/export/dqReports.xlsx
+++ b/data/export/dqReports.xlsx
@@ -63,7 +63,7 @@
     <t xml:space="preserve">Report Date (refers to the date of data export)</t>
   </si>
   <si>
-    <t xml:space="preserve">2025-03-02</t>
+    <t xml:space="preserve">2025-06-20</t>
   </si>
   <si>
     <t xml:space="preserve">dqi_co_icr</t>
@@ -489,7 +489,7 @@
     <t xml:space="preserve">pseudo_02</t>
   </si>
   <si>
-    <t xml:space="preserve">Implausible time intervall according to the mathematical ruleMR3: basis_datum=2017-05-05, basis_gebdatum=2001-05-01, min=18years, max=130years </t>
+    <t xml:space="preserve">Implausible time interval according to the mathematical rule MR3: basis_datum=2017-05-05, basis_gebdatum=2001-05-01, min=18years, max=130years </t>
   </si>
   <si>
     <t xml:space="preserve">pseudo_06</t>
@@ -501,7 +501,7 @@
     <t xml:space="preserve">Implausible combination according to the mathematical rule MR1: basis_diastol=115, basis_systol=110 </t>
   </si>
   <si>
-    <t xml:space="preserve">Implausible time intervall according to the mathematical ruleMR6: basis_exrauch=2019-01-01, basis_datum=2017-05-05, min=NAdays, max=0days </t>
+    <t xml:space="preserve">Implausible time interval according to the mathematical rule MR6: basis_exrauch=2019-01-01, basis_datum=2017-05-05, min=NAdays, max=0days </t>
   </si>
   <si>
     <t xml:space="preserve">Implausible combination according to the logical rule LR3: basis_khk=nein, basis_bypass=ja </t>
@@ -510,7 +510,7 @@
     <t xml:space="preserve">Implausible combination according to the logical rule LR3: basis_khk=nein, basis_bypass=ja</t>
   </si>
   <si>
-    <t xml:space="preserve">Implausible time intervall according to the mathematical ruleMR2: basis_datum=2017-05-20, basis_datum_blut=2017-04-27, min=-7days, max=7days </t>
+    <t xml:space="preserve">Implausible time interval according to the mathematical rule MR2: basis_datum=2017-05-20, basis_datum_blut=2017-04-27, min=-7days, max=7days </t>
   </si>
   <si>
     <t xml:space="preserve">missing_values</t>
@@ -899,11 +899,11 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1335,9 +1335,9 @@
   <dimension ref="A1:M24"/>
   <sheetFormatPr defaultColWidth="10.6796875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12.51"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="61.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="53.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="23.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="24.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="3" width="11.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="13.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="14.71"/>
@@ -1897,11 +1897,11 @@
   <dimension ref="A1:E12"/>
   <sheetFormatPr defaultColWidth="10.6796875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.96"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="61.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="51.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="28.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="23.79"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="3" width="11.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="143.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="111.97"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="6" style="1" width="9.15"/>
   </cols>
   <sheetData>
@@ -2128,11 +2128,11 @@
   <dimension ref="A1:F14"/>
   <sheetFormatPr defaultColWidth="10.6796875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12.1"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="61.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="52.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.96"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="61.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="24.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="3" width="11.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="91.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="78.72"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="69.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="7" style="1" width="9.15"/>
   </cols>
@@ -2437,8 +2437,8 @@
   <sheetFormatPr defaultColWidth="10.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="24.2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="15.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="175.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="5" style="1" width="9.15"/>
   </cols>
@@ -2534,8 +2534,7 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="13.35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="9.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="20.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="7.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="16.71"/>
@@ -3138,8 +3137,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="8.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="16.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="5.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="5.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="4.87"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="1" width="3.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="9" style="1" width="9.15"/>
   </cols>
   <sheetData>

</xml_diff>